<commit_message>
feat(mesa v3): columna CATEGORIA — reclamo/compromiso/otros por dropdown, COMENTARIO vuelve a texto libre
Detección de reclamos por CATEGORIA=reclamo en 4_pagos/efectivo y 4b_reclamos
(fallback jul-2026: COMENTARIO contiene 'reclamo' → warning; retirar en agosto).
CONCEPTO rutea plata, CATEGORIA marca eventos de mesa — no afecta montos.
Migración v2→v3 de las 7 mesas con backup (migrar_formato_v3.py, idempotente).
pagos_efectivo.xlsx pasa a 11 columnas. Docs y README sincronizados.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_5.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_5.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,8 +93,20 @@
       <color rgb="009CA3AF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00880E4F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00880E4F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -126,8 +138,13 @@
         <fgColor rgb="00FFF7ED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -149,11 +166,55 @@
         <color rgb="00FFFFFF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,6 +248,14 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -553,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -566,6 +635,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -574,16 +644,21 @@
           <t>¿Quién cobró?</t>
         </is>
       </c>
+      <c r="B1" s="12" t="n"/>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>¿Dónde vive?</t>
         </is>
       </c>
+      <c r="D1" s="12" t="n"/>
       <c r="E1" s="3" t="inlineStr">
         <is>
           <t>¿Cuánto y cuándo?</t>
         </is>
       </c>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="12" t="n"/>
       <c r="I1" s="4" t="inlineStr">
         <is>
           <t>¿Alguna nota?</t>
@@ -592,6 +667,11 @@
       <c r="J1" s="5" t="inlineStr">
         <is>
           <t>¿Qué tipo?</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué pasó?</t>
         </is>
       </c>
     </row>
@@ -644,6 +724,11 @@
       <c r="J2" s="10" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
         </is>
       </c>
     </row>
@@ -697,6 +782,11 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="K4:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="CATEGORIA inválida" error="Valores: reclamo, compromiso, otros — o dejar vacío (pago normal)." type="list">
+      <formula1>"reclamo,compromiso,otros"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -707,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -720,6 +810,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -728,16 +819,21 @@
           <t>¿Quién cobró?</t>
         </is>
       </c>
+      <c r="B1" s="12" t="n"/>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>¿Dónde vive?</t>
         </is>
       </c>
+      <c r="D1" s="12" t="n"/>
       <c r="E1" s="3" t="inlineStr">
         <is>
           <t>¿Cuánto y cuándo?</t>
         </is>
       </c>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="12" t="n"/>
       <c r="I1" s="4" t="inlineStr">
         <is>
           <t>¿Alguna nota?</t>
@@ -746,6 +842,11 @@
       <c r="J1" s="5" t="inlineStr">
         <is>
           <t>¿Qué tipo?</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué pasó?</t>
         </is>
       </c>
     </row>
@@ -798,6 +899,11 @@
       <c r="J2" s="10" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
         </is>
       </c>
     </row>
@@ -851,6 +957,11 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="K4:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="CATEGORIA inválida" error="Valores: reclamo, compromiso, otros — o dejar vacío (pago normal)." type="list">
+      <formula1>"reclamo,compromiso,otros"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -861,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -874,6 +985,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -882,16 +994,21 @@
           <t>¿Quién cobró?</t>
         </is>
       </c>
+      <c r="B1" s="12" t="n"/>
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>¿Dónde vive?</t>
         </is>
       </c>
+      <c r="D1" s="12" t="n"/>
       <c r="E1" s="3" t="inlineStr">
         <is>
           <t>¿Cuánto y cuándo?</t>
         </is>
       </c>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="13" t="n"/>
+      <c r="H1" s="12" t="n"/>
       <c r="I1" s="4" t="inlineStr">
         <is>
           <t>¿Alguna nota?</t>
@@ -900,6 +1017,11 @@
       <c r="J1" s="5" t="inlineStr">
         <is>
           <t>¿Qué tipo?</t>
+        </is>
+      </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>¿Qué pasó?</t>
         </is>
       </c>
     </row>
@@ -952,6 +1074,11 @@
       <c r="J2" s="10" t="inlineStr">
         <is>
           <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="inlineStr">
+        <is>
+          <t>CATEGORIA</t>
         </is>
       </c>
     </row>
@@ -1005,6 +1132,11 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="E1:H1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="K4:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="CATEGORIA inválida" error="Valores: reclamo, compromiso, otros — o dejar vacío (pago normal)." type="list">
+      <formula1>"reclamo,compromiso,otros"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>